<commit_message>
Show variable costs on the workbook's Dashboard sheet
The live Excel view now breaks contribution margin down to what remains after
shipping, fulfilment, payment fees and advertising. Formulas follow the
Settings inputs, sit in D9:E17 clear of the charts, and round shipping per
order like the pipeline.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/unit-economics-input.xlsx
+++ b/assets/unit-economics-input.xlsx
@@ -431,8 +431,8 @@
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="4" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
@@ -508,6 +508,17 @@
           <t xml:space="preserve">Value</t>
         </is>
       </c>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">After variable costs</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -519,6 +530,16 @@
         <f>SUMPRODUCT(('Orders'!$E$3:$E$1200*'Orders'!$G$3:$G$1200)-'Orders'!$H$3:$H$1200)</f>
         <v>83755.43</v>
       </c>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contribution margin</t>
+        </is>
+      </c>
+      <c r="E10" s="6">
+        <f>B11</f>
+        <v>51319.39</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -530,6 +551,16 @@
         <f>SUM(E27:E33)</f>
         <v>51319.39</v>
       </c>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+ Shipping charged ex VAT</t>
+        </is>
+      </c>
+      <c r="E11" s="6">
+        <f>ROUND(ROUND('Settings'!B13/(1+'Settings'!B6/100),2)*SUMPRODUCT(1/COUNTIF('Orders'!$A$3:$A$1200,'Orders'!$A$3:$A$1200)),2)</f>
+        <v>2174.04</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -541,6 +572,16 @@
         <f>COUNTA('Orders'!$A$3:$A$1200)</f>
         <v>1198</v>
       </c>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- Fulfilment</t>
+        </is>
+      </c>
+      <c r="E12" s="6">
+        <f>ROUND('Settings'!B12*SUMPRODUCT(1/COUNTIF('Orders'!$A$3:$A$1200,'Orders'!$A$3:$A$1200)),2)</f>
+        <v>4811.4</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -552,9 +593,30 @@
         <f>SUM('Orders'!$G$3:$G$1200)</f>
         <v>1358</v>
       </c>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- Payment fees</t>
+        </is>
+      </c>
+      <c r="E13" s="6">
+        <f>ROUND('Settings'!B14/100*(B10+'Settings'!B13*SUMPRODUCT(1/COUNTIF('Orders'!$A$3:$A$1200,'Orders'!$A$3:$A$1200)))+'Settings'!B15*SUMPRODUCT(1/COUNTIF('Orders'!$A$3:$A$1200,'Orders'!$A$3:$A$1200)),2)</f>
+        <v>1518.51</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">- Advertising</t>
+        </is>
+      </c>
+      <c r="E14" s="6">
+        <f>SUM('Settings'!$B$19:$B$60)</f>
+        <v>11997</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
@@ -566,6 +628,16 @@
         <is>
           <t xml:space="preserve">Value</t>
         </is>
+      </c>
+      <c r="C15" s="1"/>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">After variable costs</t>
+        </is>
+      </c>
+      <c r="E15" s="11">
+        <f>E10+E11-E12-E13-E14</f>
+        <v>35166.52</v>
       </c>
     </row>
     <row r="16">
@@ -578,6 +650,16 @@
         <f>'Settings'!B8</f>
         <v>100000</v>
       </c>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Share of net sales</t>
+        </is>
+      </c>
+      <c r="E16" s="7">
+        <f>IF(SUM('Orders'!$I$3:$I$1200)=0,0,E15/SUM('Orders'!$I$3:$I$1200))</f>
+        <v>0.508</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -589,6 +671,13 @@
         <f>B10/B16</f>
         <v>0.8376</v>
       </c>
+      <c r="C17" s="5"/>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Costs come from Settings. Not net profit.</t>
+        </is>
+      </c>
+      <c r="E17" s="5"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -939,7 +1028,7 @@
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Live, formula-driven Excel companion. The polished interactive dashboard is online.</t>
+          <t xml:space="preserve">Live, formula-driven Excel companion, including what remains after variable costs. The polished interactive dashboard is online.</t>
         </is>
       </c>
     </row>

</xml_diff>